<commit_message>
Release 0.8.8 action presentation, kong fixes and compact Telegram reports
</commit_message>
<xml_diff>
--- a/server/report-xlsx/templates/dailyScore.xlsx
+++ b/server/report-xlsx/templates/dailyScore.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="日结" sheetId="1" r:id="R91263d0c1d564289"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="日结" sheetId="1" r:id="R0e003002f0784467"/>
   </sheets>
 </workbook>
 </file>
@@ -65,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -100,6 +100,9 @@
     </xf>
     <xf numFmtId="201" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -303,29 +306,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="15" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="str">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="13" t="str">
         <v>日结算表 2026.9.16</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="7" t="str">
         <v>战队名</v>
       </c>
@@ -351,7 +354,7 @@
         <v>总结算</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="8"/>

</xml_diff>